<commit_message>
Microsoft Office fixtures re-saved after the rename; last ox leftovers fixed
- examples/hello-table/fixtures/*.msoffice-flow-*: the maintainer's seven saves (Excel 16.03, Word and
  PowerPoint 16.0 for Mac) from fresh Demo B exports; last-modified-by Milleleaf, folder path
  trimmed to ~/.
- run.sh and tools/inventory/roundtrip.sh called target/debug/ox; the binary is now mleaf.
- README, model.rs and schema/mleaf.tsp still named schema/ox.tsp.

Box: Rust tests 192 passed, 0 failed, 9 ignored; run.sh steps 1-19 exit 0; site build, CSP,
typecheck, check, check-compare, check-privacy and check-flow exit 0.
</commit_message>
<xml_diff>
--- a/examples/hello-table/fixtures/finance.msoffice-flow-edited.xlsx
+++ b/examples/hello-table/fixtures/finance.msoffice-flow-edited.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/examples/hello-table/fixtures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="~/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC7EB695-9016-904A-A59D-E6F92BA615BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4354DC61-1DE5-EE46-8C32-5793FB2EA9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,11 +16,11 @@
     <sheet name="Q3" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ox_3f1c2a90_0000_4c1e_9a00_000000000011" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000011">'Q3'!$A$1</definedName>
-    <definedName name="ox_3f1c2a90_0000_4c1e_9a00_000000000012" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000012">'Q3'!$A$1:$B$4</definedName>
-    <definedName name="ox_3f1c2a90_0000_4c1e_9a00_000000000013" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000013">'Q3'!$B$5</definedName>
-    <definedName name="ox_revision">"291ed7b7723c8bc826a4ab9b"</definedName>
-    <definedName name="ox_workbook">"3f1c2a90-0000-4c1e-9a00-000000000010"</definedName>
+    <definedName name="mleaf_3f1c2a90_0000_4c1e_9a00_000000000011" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000011">'Q3'!$A$1</definedName>
+    <definedName name="mleaf_3f1c2a90_0000_4c1e_9a00_000000000012" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000012">'Q3'!$A$1:$B$4</definedName>
+    <definedName name="mleaf_3f1c2a90_0000_4c1e_9a00_000000000013" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000013">'Q3'!$B$5</definedName>
+    <definedName name="mleaf_revision">"291ed7b7723c8bc826a4ab9b"</definedName>
+    <definedName name="mleaf_workbook">"3f1c2a90-0000-4c1e-9a00-000000000010"</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>